<commit_message>
[KGDB][ETHER] - update src with reduced 'phy_start'
</commit_message>
<xml_diff>
--- a/03_Learning/04_LINUX_Common/04_Modules/BBB_KGDB/11_ETHERNET/03_DEBUG/CUSTOM/BBB.xlsx
+++ b/03_Learning/04_LINUX_Common/04_Modules/BBB_KGDB/11_ETHERNET/03_DEBUG/CUSTOM/BBB.xlsx
@@ -344,16 +344,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -455,7 +451,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:U34"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="36.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="17.33"/>
@@ -477,7 +473,6 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="2"/>
       <c r="F1" s="1" t="s">
         <v>1</v>
       </c>
@@ -498,47 +493,47 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3" t="s">
+      <c r="H2" s="2"/>
+      <c r="I2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="J2" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="K2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="L2" s="3" t="s">
+      <c r="L2" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="M2" s="3" t="s">
+      <c r="M2" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="N2" s="3" t="s">
+      <c r="N2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="O2" s="3" t="s">
+      <c r="O2" s="2" t="s">
         <v>20</v>
       </c>
     </row>
@@ -556,29 +551,29 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
-      <c r="J5" s="4"/>
-      <c r="K5" s="4"/>
-      <c r="L5" s="4"/>
-      <c r="M5" s="4"/>
-      <c r="N5" s="4"/>
-      <c r="O5" s="4"/>
-      <c r="P5" s="4"/>
-      <c r="Q5" s="4"/>
-      <c r="R5" s="4"/>
-      <c r="S5" s="4"/>
-      <c r="T5" s="4"/>
-      <c r="U5" s="4"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+      <c r="L5" s="3"/>
+      <c r="M5" s="3"/>
+      <c r="N5" s="3"/>
+      <c r="O5" s="3"/>
+      <c r="P5" s="3"/>
+      <c r="Q5" s="3"/>
+      <c r="R5" s="3"/>
+      <c r="S5" s="3"/>
+      <c r="T5" s="3"/>
+      <c r="U5" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
@@ -592,29 +587,29 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B8" s="4"/>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
-      <c r="F8" s="4"/>
-      <c r="G8" s="4"/>
-      <c r="H8" s="4"/>
-      <c r="I8" s="4"/>
-      <c r="J8" s="4"/>
-      <c r="K8" s="4"/>
-      <c r="L8" s="4"/>
-      <c r="M8" s="4"/>
-      <c r="N8" s="4"/>
-      <c r="O8" s="4"/>
-      <c r="P8" s="4"/>
-      <c r="Q8" s="4"/>
-      <c r="R8" s="4"/>
-      <c r="S8" s="4"/>
-      <c r="T8" s="4"/>
-      <c r="U8" s="4"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3"/>
+      <c r="L8" s="3"/>
+      <c r="M8" s="3"/>
+      <c r="N8" s="3"/>
+      <c r="O8" s="3"/>
+      <c r="P8" s="3"/>
+      <c r="Q8" s="3"/>
+      <c r="R8" s="3"/>
+      <c r="S8" s="3"/>
+      <c r="T8" s="3"/>
+      <c r="U8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
@@ -622,29 +617,29 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4"/>
-      <c r="H10" s="4"/>
-      <c r="I10" s="4"/>
-      <c r="J10" s="4"/>
-      <c r="K10" s="4"/>
-      <c r="L10" s="4"/>
-      <c r="M10" s="4"/>
-      <c r="N10" s="4"/>
-      <c r="O10" s="4"/>
-      <c r="P10" s="4"/>
-      <c r="Q10" s="4"/>
-      <c r="R10" s="4"/>
-      <c r="S10" s="4"/>
-      <c r="T10" s="4"/>
-      <c r="U10" s="4"/>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
+      <c r="J10" s="3"/>
+      <c r="K10" s="3"/>
+      <c r="L10" s="3"/>
+      <c r="M10" s="3"/>
+      <c r="N10" s="3"/>
+      <c r="O10" s="3"/>
+      <c r="P10" s="3"/>
+      <c r="Q10" s="3"/>
+      <c r="R10" s="3"/>
+      <c r="S10" s="3"/>
+      <c r="T10" s="3"/>
+      <c r="U10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
@@ -706,7 +701,7 @@
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="5" t="s">
+      <c r="A21" s="4" t="s">
         <v>39</v>
       </c>
       <c r="F21" s="0" t="s">
@@ -738,10 +733,10 @@
       <c r="H25" s="0" t="s">
         <v>45</v>
       </c>
-      <c r="L25" s="6" t="s">
+      <c r="L25" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="O25" s="7" t="s">
+      <c r="O25" s="6" t="s">
         <v>47</v>
       </c>
     </row>
@@ -752,7 +747,7 @@
       <c r="L26" s="0" t="s">
         <v>49</v>
       </c>
-      <c r="O26" s="7"/>
+      <c r="O26" s="6"/>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H27" s="0" t="s">
@@ -761,7 +756,7 @@
       <c r="L27" s="0" t="s">
         <v>51</v>
       </c>
-      <c r="O27" s="7"/>
+      <c r="O27" s="6"/>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H28" s="0" t="s">
@@ -780,12 +775,12 @@
       <c r="G30" s="0" t="s">
         <v>55</v>
       </c>
-      <c r="H30" s="6" t="s">
+      <c r="H30" s="5" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="0" t="s">
+      <c r="A31" s="4" t="s">
         <v>57</v>
       </c>
       <c r="I31" s="0" t="s">
@@ -798,7 +793,7 @@
       </c>
     </row>
     <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="0" t="s">
+      <c r="A33" s="4" t="s">
         <v>60</v>
       </c>
       <c r="I33" s="0" t="s">
@@ -812,24 +807,24 @@
       </c>
     </row>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="4" t="s">
+      <c r="A34" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B34" s="4"/>
-      <c r="C34" s="4"/>
-      <c r="D34" s="4"/>
-      <c r="E34" s="4"/>
-      <c r="F34" s="4"/>
-      <c r="G34" s="4"/>
-      <c r="H34" s="4"/>
-      <c r="I34" s="4"/>
-      <c r="J34" s="4"/>
-      <c r="K34" s="4"/>
-      <c r="L34" s="4"/>
-      <c r="M34" s="4"/>
-      <c r="N34" s="4"/>
-      <c r="O34" s="4"/>
-      <c r="P34" s="4"/>
+      <c r="B34" s="3"/>
+      <c r="C34" s="3"/>
+      <c r="D34" s="3"/>
+      <c r="E34" s="3"/>
+      <c r="F34" s="3"/>
+      <c r="G34" s="3"/>
+      <c r="H34" s="3"/>
+      <c r="I34" s="3"/>
+      <c r="J34" s="3"/>
+      <c r="K34" s="3"/>
+      <c r="L34" s="3"/>
+      <c r="M34" s="3"/>
+      <c r="N34" s="3"/>
+      <c r="O34" s="3"/>
+      <c r="P34" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>